<commit_message>
app works with new file. Bringing in as xlsx for easier read-in
</commit_message>
<xml_diff>
--- a/data/antennaMetadata.xlsx
+++ b/data/antennaMetadata.xlsx
@@ -48,31 +48,31 @@
     <t>0B</t>
   </si>
   <si>
-    <t>01</t>
-  </si>
-  <si>
-    <t>02</t>
-  </si>
-  <si>
-    <t>03</t>
-  </si>
-  <si>
-    <t>04</t>
-  </si>
-  <si>
-    <t>05</t>
-  </si>
-  <si>
-    <t>06</t>
-  </si>
-  <si>
-    <t>07</t>
-  </si>
-  <si>
-    <t>08</t>
-  </si>
-  <si>
-    <t>09</t>
+    <t>1</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>9</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
updated to use csvs and metadata tweaked to comply
</commit_message>
<xml_diff>
--- a/data/antennaMetadata.xlsx
+++ b/data/antennaMetadata.xlsx
@@ -48,31 +48,31 @@
     <t>0B</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>9</t>
+    <t>01</t>
+  </si>
+  <si>
+    <t>02</t>
+  </si>
+  <si>
+    <t>03</t>
+  </si>
+  <si>
+    <t>04</t>
+  </si>
+  <si>
+    <t>05</t>
+  </si>
+  <si>
+    <t>06</t>
+  </si>
+  <si>
+    <t>07</t>
+  </si>
+  <si>
+    <t>08</t>
+  </si>
+  <si>
+    <t>09</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
changed status function to reflect last of day more accurately. cleanup
</commit_message>
<xml_diff>
--- a/data/antennaMetadata.xlsx
+++ b/data/antennaMetadata.xlsx
@@ -18,6 +18,64 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Graf, Sam</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Graf, Sam:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+corresponds to names of antennas coming off the detection file. If they change, this needs to change too</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Graf, Sam:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+turning each antenna number into US/DS array</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="18">
   <si>
@@ -79,7 +137,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -213,6 +271,19 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="33">
@@ -879,7 +950,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1059,5 +1130,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>